<commit_message>
Translate columns, labels, and scripts to English for the public portfolio.
</commit_message>
<xml_diff>
--- a/matlab/results/dataset_summary.xlsx
+++ b/matlab/results/dataset_summary.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="114" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="152" uniqueCount="40">
   <si>
     <t>Variable</t>
   </si>
@@ -82,6 +82,57 @@
   </si>
   <si>
     <t>Missing</t>
+  </si>
+  <si>
+    <t>Order_ID</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Sales_Channel</t>
+  </si>
+  <si>
+    <t>Customer_Type</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Unit_Price_TL</t>
+  </si>
+  <si>
+    <t>Discount_Rate</t>
+  </si>
+  <si>
+    <t>Unit_Cost_TL</t>
+  </si>
+  <si>
+    <t>Payment_Method</t>
+  </si>
+  <si>
+    <t>Net_Sales</t>
+  </si>
+  <si>
+    <t>Total_Cost</t>
+  </si>
+  <si>
+    <t>Profit</t>
+  </si>
+  <si>
+    <t>Profit_Margin</t>
   </si>
 </sst>
 </file>
@@ -130,7 +181,7 @@
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" customWidth="true"/>
+    <col min="1" max="1" width="17" customWidth="true"/>
     <col min="2" max="2" width="7.42578125" customWidth="true"/>
     <col min="3" max="3" width="13.5703125" customWidth="true"/>
     <col min="4" max="4" width="7.85546875" customWidth="true"/>
@@ -152,7 +203,7 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="B2" s="0" t="s">
         <v>19</v>
@@ -166,7 +217,7 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="B3" s="0" t="s">
         <v>19</v>
@@ -180,7 +231,7 @@
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="B4" s="0" t="s">
         <v>19</v>
@@ -194,7 +245,7 @@
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="B5" s="0" t="s">
         <v>19</v>
@@ -208,7 +259,7 @@
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="B6" s="0" t="s">
         <v>19</v>
@@ -222,7 +273,7 @@
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="B7" s="0" t="s">
         <v>19</v>
@@ -236,7 +287,7 @@
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="B8" s="0" t="s">
         <v>19</v>
@@ -250,7 +301,7 @@
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="B9" s="0" t="s">
         <v>19</v>
@@ -264,7 +315,7 @@
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="B10" s="0" t="s">
         <v>20</v>
@@ -278,7 +329,7 @@
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>20</v>
@@ -292,7 +343,7 @@
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="B12" s="0" t="s">
         <v>20</v>
@@ -306,7 +357,7 @@
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="B13" s="0" t="s">
         <v>20</v>
@@ -320,7 +371,7 @@
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="B14" s="0" t="s">
         <v>19</v>
@@ -334,7 +385,7 @@
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="B15" s="0" t="s">
         <v>20</v>
@@ -348,7 +399,7 @@
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="B16" s="0" t="s">
         <v>20</v>
@@ -362,7 +413,7 @@
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="B17" s="0" t="s">
         <v>20</v>
@@ -374,7 +425,7 @@
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="B18" s="0" t="s">
         <v>20</v>

</xml_diff>